<commit_message>
feat(users) : - add phone number & photo
</commit_message>
<xml_diff>
--- a/public/excel/Template Pengguna.xlsx
+++ b/public/excel/Template Pengguna.xlsx
@@ -11,72 +11,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
   <si>
     <t>User Name</t>
   </si>
   <si>
-    <t>Kode RBM</t>
-  </si>
-  <si>
-    <t>Nama</t>
-  </si>
-  <si>
-    <t>No. Hp</t>
-  </si>
-  <si>
-    <t>Tipe</t>
-  </si>
-  <si>
-    <t>Jabatan</t>
+    <t>doni</t>
+  </si>
+  <si>
+    <t>DNS</t>
+  </si>
+  <si>
+    <t>Doni Setiawan</t>
+  </si>
+  <si>
+    <t>0811345345</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>dona</t>
+  </si>
+  <si>
+    <t>DNY</t>
+  </si>
+  <si>
+    <t>Dona Yunita</t>
+  </si>
+  <si>
+    <t>0811678678</t>
   </si>
   <si>
     <t>UID</t>
-  </si>
-  <si>
-    <t>UP3</t>
-  </si>
-  <si>
-    <t>ULP</t>
-  </si>
-  <si>
-    <t>Kode Hak Akses</t>
-  </si>
-  <si>
-    <t>doni</t>
-  </si>
-  <si>
-    <t>DNS</t>
-  </si>
-  <si>
-    <t>Doni Setiawan</t>
-  </si>
-  <si>
-    <t>0811345345</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>dona</t>
-  </si>
-  <si>
-    <t>DNY</t>
-  </si>
-  <si>
-    <t>Dona Yunita</t>
-  </si>
-  <si>
-    <t>0811678678</t>
-  </si>
-  <si>
-    <t>Petugas</t>
   </si>
   <si>
     <t>Staff</t>
@@ -394,51 +367,51 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G2" s="2">
         <v>17.0</v>
@@ -450,27 +423,27 @@
         <v>17100.0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2">
         <v>17.0</v>
@@ -482,7 +455,7 @@
         <v>17100.0</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
order upload, baru bs upload, blm ada log dll
</commit_message>
<xml_diff>
--- a/public/excel/Template Pengguna.xlsx
+++ b/public/excel/Template Pengguna.xlsx
@@ -1,17 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ardiyanto/Program/pratul-online/public/excel/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B7CA91E-130B-7742-B57C-7A7A25A4494A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>User Name</t>
   </si>
@@ -28,12 +45,6 @@
     <t>0811345345</t>
   </si>
   <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -56,41 +67,81 @@
   </si>
   <si>
     <t>U2</t>
+  </si>
+  <si>
+    <t>NO HP</t>
+  </si>
+  <si>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Tipe</t>
+  </si>
+  <si>
+    <t>ULP</t>
+  </si>
+  <si>
+    <t>Petugas</t>
+  </si>
+  <si>
+    <t>Jabatan</t>
+  </si>
+  <si>
+    <t>UP3</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>U1 untuk Admin</t>
+  </si>
+  <si>
+    <t>U2 untuk Petugas</t>
+  </si>
+  <si>
+    <t>RBM</t>
+  </si>
+  <si>
+    <t>isi UID, UP2K,UP2D,UP3,ULP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8.0"/>
+      <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF0B4CB4"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF0B4CB4"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -101,7 +152,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -111,7 +162,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -125,44 +182,40 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -352,49 +405,52 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -408,57 +464,57 @@
         <v>4</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="2">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2">
+        <v>17171</v>
+      </c>
+      <c r="I2" s="2">
+        <v>17100</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="2">
-        <v>17.0</v>
-      </c>
-      <c r="H2" s="2">
-        <v>17171.0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>17100.0</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2">
+        <v>17</v>
+      </c>
+      <c r="H3" s="2">
+        <v>17171</v>
+      </c>
+      <c r="I3" s="2">
+        <v>17100</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2">
-        <v>17.0</v>
-      </c>
-      <c r="H3" s="2">
-        <v>17171.0</v>
-      </c>
-      <c r="I3" s="2">
-        <v>17100.0</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4">
+    </row>
+    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -470,7 +526,7 @@
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -482,7 +538,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -494,7 +550,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -506,7 +562,7 @@
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -518,7 +574,7 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -530,7 +586,7 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -542,7 +598,33 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
     </row>
+    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>